<commit_message>
Quitar categorias, paginacion server-side, ganancias y entorno Docker
- Eliminar por completo categorias y subcategorias (BD, modelos, vistas, rutas, imports/exports)
- Campo de ganancias en ventas y detalle de venta (+ PDF, Excel y dashboard)
- Paginacion server-side y buscador en todos los listados (rendimiento con +2000 productos)
- Marca y unidad de medida opcionales en productos
- Filtro por rango de fechas con totales de ventas y ganancias
- Dockerizacion funcional: entrypoint con migraciones/seed, healthcheck de MySQL y .env.docker
- NIT configurable por variable de entorno
- Varios arreglos de UI y de datos

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/storage/app/public/template/planilla_importar_productos.xlsx
+++ b/storage/app/public/template/planilla_importar_productos.xlsx
@@ -1,42 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27531"/>
-  <workbookPr defaultThemeVersion="202300"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\user\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{7BFCECD4-018B-4CE3-A1FA-09E6EBC7562A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView xWindow="12120" yWindow="3900" windowWidth="21600" windowHeight="11385" xr2:uid="{C8853B33-AF5B-43A5-860D-23A923F8BAA0}"/>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja1" sheetId="1" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
-      <x15:workbookPr chartTrackingRefBase="1"/>
-    </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="7">
   <si>
     <t>nombre_producto</t>
   </si>
@@ -51,12 +30,6 @@
   </si>
   <si>
     <t>precio_venta</t>
-  </si>
-  <si>
-    <t>nombre_subcategoria</t>
-  </si>
-  <si>
-    <t>id_categoria</t>
   </si>
   <si>
     <t>id_marca</t>
@@ -68,20 +41,27 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
+  <fonts count="2">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Consolas"/>
-      <family val="3"/>
     </font>
   </fonts>
   <fills count="2">
@@ -105,30 +85,22 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="3">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
+    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="1">
+      <alignment vertical="center" textRotation="0" wrapText="false" shrinkToFit="false"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -170,7 +142,7 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Aptos Display" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Display"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック Light"/>
@@ -222,7 +194,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Aptos Narrow" panose="02110004020202020204"/>
+        <a:latin typeface="Aptos Narrow"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
         <a:font script="Jpan" typeface="游ゴシック"/>
@@ -283,182 +255,187 @@
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:lumMod val="110000"/>
-                <a:satMod val="105000"/>
-                <a:tint val="67000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="103000"/>
-                <a:tint val="73000"/>
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="105000"/>
-                <a:satMod val="109000"/>
-                <a:tint val="81000"/>
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="1"/>
         </a:gradFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:satMod val="103000"/>
-                <a:lumMod val="102000"/>
-                <a:tint val="94000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:satMod val="110000"/>
-                <a:lumMod val="100000"/>
-                <a:shade val="100000"/>
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:lumMod val="99000"/>
-                <a:satMod val="120000"/>
-                <a:shade val="78000"/>
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:lin ang="16200000" scaled="0"/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
-        <a:ln w="12700" cap="flat" cmpd="sng" algn="ctr">
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
-            <a:schemeClr val="phClr"/>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
-        </a:ln>
-        <a:ln w="19050" cap="flat" cmpd="sng" algn="ctr">
-          <a:solidFill>
-            <a:schemeClr val="phClr"/>
-          </a:solidFill>
-          <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
         </a:ln>
         <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
           <a:solidFill>
             <a:schemeClr val="phClr"/>
           </a:solidFill>
           <a:prstDash val="solid"/>
-          <a:miter lim="800000"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
         </a:ln>
       </a:lnStyleLst>
       <a:effectStyleLst>
         <a:effectStyle>
-          <a:effectLst/>
-        </a:effectStyle>
-        <a:effectStyle>
-          <a:effectLst/>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
         </a:effectStyle>
         <a:effectStyle>
           <a:effectLst>
-            <a:outerShdw blurRad="57150" dist="19050" dir="5400000" algn="ctr" rotWithShape="0">
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
               <a:srgbClr val="000000">
-                <a:alpha val="63000"/>
+                <a:alpha val="35000"/>
               </a:srgbClr>
             </a:outerShdw>
           </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
         </a:effectStyle>
       </a:effectStyleLst>
       <a:bgFillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
         </a:solidFill>
-        <a:solidFill>
-          <a:schemeClr val="phClr">
-            <a:tint val="95000"/>
-            <a:satMod val="170000"/>
-          </a:schemeClr>
-        </a:solidFill>
         <a:gradFill rotWithShape="1">
           <a:gsLst>
             <a:gs pos="0">
               <a:schemeClr val="phClr">
-                <a:tint val="93000"/>
-                <a:satMod val="150000"/>
-                <a:shade val="98000"/>
-                <a:lumMod val="102000"/>
-              </a:schemeClr>
-            </a:gs>
-            <a:gs pos="50000">
-              <a:schemeClr val="phClr">
-                <a:tint val="98000"/>
-                <a:satMod val="130000"/>
-                <a:shade val="90000"/>
-                <a:lumMod val="103000"/>
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
               </a:schemeClr>
             </a:gs>
             <a:gs pos="100000">
               <a:schemeClr val="phClr">
-                <a:shade val="63000"/>
-                <a:satMod val="120000"/>
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
               </a:schemeClr>
             </a:gs>
           </a:gsLst>
-          <a:lin ang="5400000" scaled="0"/>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults>
-    <a:lnDef>
-      <a:spPr/>
-      <a:bodyPr/>
-      <a:lstStyle/>
-      <a:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </a:style>
-    </a:lnDef>
-  </a:objectDefaults>
+  <a:objectDefaults/>
   <a:extraClrSchemeLst/>
-  <a:extLst>
-    <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{2E142A2C-CD16-42D6-873A-C26D2A0506FA}" vid="{1BDDFF52-6CD6-40A5-AB3C-68EB2F1E4D0A}"/>
-    </a:ext>
-  </a:extLst>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4B41348E-6CF0-4FC3-8F66-247E0F09294B}">
-  <dimension ref="A1:I1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:G1"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="24.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="21.85546875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="28.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="23" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.28515625" customWidth="true" style="0"/>
+    <col min="2" max="2" width="24.140625" customWidth="true" style="0"/>
+    <col min="3" max="3" width="21.85546875" customWidth="true" style="0"/>
+    <col min="4" max="4" width="28.85546875" customWidth="true" style="0"/>
+    <col min="5" max="5" width="14.7109375" customWidth="true" style="0"/>
+    <col min="6" max="6" width="10.140625" customWidth="true" style="0"/>
+    <col min="7" max="7" width="19.42578125" customWidth="true" style="0"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" s="2" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -480,14 +457,19 @@
       <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
     </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>